<commit_message>
Update MLB weather 2026-07-27 12:14 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v5_2026_07_27.xlsx
+++ b/mlb_weather_professional_v5_2026_07_27.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1692" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1692" uniqueCount="365">
   <si>
     <t>Date</t>
   </si>
@@ -551,40 +551,37 @@
     <t>HIGH</t>
   </si>
   <si>
-    <t>2026-07-27 12:09:51 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:09:52 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:09:54 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:09:55 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:09:56 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:09:58 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:09:59 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:10:04 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:10:05 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:10:07 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:10:10 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:10:12 PM PDT</t>
+    <t>2026-07-27 12:14:09 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:14:10 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:14:11 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:14:12 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:14:13 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:14:14 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:14:15 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:14:16 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:14:17 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:14:18 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:14:19 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -965,40 +962,37 @@
     <t>09:45 PM PDT</t>
   </si>
   <si>
-    <t>2026-07-27 19:09:51 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:09:52 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:09:54 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:09:55 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:09:56 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:09:58 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:09:59 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:10:04 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:10:05 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:10:07 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:10:10 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:10:12 UTC</t>
+    <t>2026-07-27 19:14:09 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:14:10 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:14:11 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:14:12 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:14:13 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:14:14 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:14:15 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:14:16 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:14:17 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:14:18 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:14:19 UTC</t>
   </si>
   <si>
     <t>2026-07-27T18:26:57+00:00</t>
@@ -1862,7 +1856,7 @@
         <v>0</v>
       </c>
       <c r="AC2">
-        <v>93</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="AD2" t="s">
         <v>164</v>
@@ -1931,7 +1925,7 @@
         <v>176</v>
       </c>
       <c r="AZ2">
-        <v>42.9</v>
+        <v>47.2</v>
       </c>
       <c r="BA2">
         <v>5</v>
@@ -2065,7 +2059,7 @@
         <v>167</v>
       </c>
       <c r="AR3">
-        <v>-3</v>
+        <v>-2.6</v>
       </c>
       <c r="AS3">
         <v>0</v>
@@ -2089,7 +2083,7 @@
         <v>177</v>
       </c>
       <c r="AZ3">
-        <v>20.7</v>
+        <v>25</v>
       </c>
       <c r="BA3">
         <v>5</v>
@@ -2223,7 +2217,7 @@
         <v>168</v>
       </c>
       <c r="AR4">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="AS4">
         <v>0</v>
@@ -2247,7 +2241,7 @@
         <v>178</v>
       </c>
       <c r="AZ4">
-        <v>48.3</v>
+        <v>52.6</v>
       </c>
       <c r="BA4">
         <v>5</v>
@@ -2381,7 +2375,7 @@
         <v>168</v>
       </c>
       <c r="AR5">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="AS5">
         <v>0</v>
@@ -2405,7 +2399,7 @@
         <v>179</v>
       </c>
       <c r="AZ5">
-        <v>38.1</v>
+        <v>42.4</v>
       </c>
       <c r="BA5">
         <v>5</v>
@@ -2536,10 +2530,10 @@
         <v>67.8</v>
       </c>
       <c r="AQ6" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="AR6">
-        <v>6.6</v>
+        <v>3.9</v>
       </c>
       <c r="AS6">
         <v>0</v>
@@ -2563,7 +2557,7 @@
         <v>180</v>
       </c>
       <c r="AZ6">
-        <v>46.4</v>
+        <v>50.7</v>
       </c>
       <c r="BA6">
         <v>5</v>
@@ -2697,7 +2691,7 @@
         <v>168</v>
       </c>
       <c r="AR7">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="AS7">
         <v>0</v>
@@ -2718,10 +2712,10 @@
         <v>19.2</v>
       </c>
       <c r="AY7" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AZ7">
-        <v>137.2</v>
+        <v>141.4</v>
       </c>
       <c r="BA7">
         <v>5</v>
@@ -2855,7 +2849,7 @@
         <v>169</v>
       </c>
       <c r="AR8">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="AS8">
         <v>0</v>
@@ -2876,10 +2870,10 @@
         <v>14.1</v>
       </c>
       <c r="AY8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AZ8">
-        <v>18.3</v>
+        <v>22.6</v>
       </c>
       <c r="BA8">
         <v>5</v>
@@ -3010,10 +3004,10 @@
         <v>85.09999999999999</v>
       </c>
       <c r="AQ9" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AR9">
-        <v>3.2</v>
+        <v>-1.6</v>
       </c>
       <c r="AS9">
         <v>0</v>
@@ -3034,10 +3028,10 @@
         <v>36.2</v>
       </c>
       <c r="AY9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AZ9">
-        <v>48.9</v>
+        <v>53.1</v>
       </c>
       <c r="BA9">
         <v>5</v>
@@ -3171,7 +3165,7 @@
         <v>169</v>
       </c>
       <c r="AR10">
-        <v>5.7</v>
+        <v>5.4</v>
       </c>
       <c r="AS10">
         <v>0</v>
@@ -3192,10 +3186,10 @@
         <v>9.6</v>
       </c>
       <c r="AY10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AZ10">
-        <v>18.4</v>
+        <v>22.6</v>
       </c>
       <c r="BA10">
         <v>5</v>
@@ -3329,7 +3323,7 @@
         <v>169</v>
       </c>
       <c r="AR11">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="AS11">
         <v>0</v>
@@ -3350,10 +3344,10 @@
         <v>13.5</v>
       </c>
       <c r="AY11" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AZ11">
-        <v>40.4</v>
+        <v>44.6</v>
       </c>
       <c r="BA11">
         <v>5</v>
@@ -3508,10 +3502,10 @@
         <v>5.3</v>
       </c>
       <c r="AY12" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AZ12">
-        <v>38.9</v>
+        <v>43</v>
       </c>
       <c r="BA12">
         <v>5</v>
@@ -3645,7 +3639,7 @@
         <v>169</v>
       </c>
       <c r="AR13">
-        <v>4.6</v>
+        <v>5.1</v>
       </c>
       <c r="AS13">
         <v>0</v>
@@ -3666,10 +3660,10 @@
         <v>9.800000000000001</v>
       </c>
       <c r="AY13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AZ13">
-        <v>38.4</v>
+        <v>42.5</v>
       </c>
       <c r="BA13">
         <v>5</v>
@@ -3810,286 +3804,286 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>190</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>50</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>51</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>52</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="BI1" s="1" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="BJ1" s="1" t="s">
+      <c r="BK1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="BK1" s="1" t="s">
+      <c r="BL1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="BL1" s="1" t="s">
+      <c r="BM1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="BM1" s="1" t="s">
+      <c r="BN1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="BN1" s="1" t="s">
+      <c r="BO1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="BO1" s="1" t="s">
+      <c r="BP1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="BP1" s="1" t="s">
+      <c r="BQ1" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="BQ1" s="1" t="s">
+      <c r="BR1" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="BR1" s="1" t="s">
+      <c r="BS1" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="BS1" s="1" t="s">
+      <c r="BT1" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="BT1" s="1" t="s">
+      <c r="BU1" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="BU1" s="1" t="s">
+      <c r="BV1" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="BV1" s="1" t="s">
+      <c r="BW1" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="BW1" s="1" t="s">
+      <c r="BX1" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="BX1" s="1" t="s">
+      <c r="BY1" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="BY1" s="1" t="s">
+      <c r="BZ1" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="BZ1" s="1" t="s">
+      <c r="CA1" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="CA1" s="1" t="s">
+      <c r="CB1" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="CB1" s="1" t="s">
+      <c r="CC1" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="CC1" s="1" t="s">
+      <c r="CD1" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="CD1" s="1" t="s">
+      <c r="CE1" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="CE1" s="1" t="s">
+      <c r="CF1" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="CF1" s="1" t="s">
+      <c r="CG1" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="CG1" s="1" t="s">
+      <c r="CH1" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="CH1" s="1" t="s">
+      <c r="CI1" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="CI1" s="1" t="s">
+      <c r="CJ1" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="CJ1" s="1" t="s">
+      <c r="CK1" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="CK1" s="1" t="s">
+      <c r="CL1" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="CL1" s="1" t="s">
+      <c r="CM1" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="CM1" s="1" t="s">
+      <c r="CN1" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="CN1" s="1" t="s">
+      <c r="CO1" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="CO1" s="1" t="s">
+      <c r="CP1" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="CP1" s="1" t="s">
+      <c r="CQ1" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="CQ1" s="1" t="s">
+      <c r="CR1" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="CR1" s="1" t="s">
+      <c r="CS1" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="CS1" s="1" t="s">
+      <c r="CT1" s="1" t="s">
         <v>277</v>
-      </c>
-      <c r="CT1" s="1" t="s">
-        <v>278</v>
       </c>
       <c r="CU1" s="1" t="s">
         <v>49</v>
@@ -4098,16 +4092,16 @@
         <v>48</v>
       </c>
       <c r="CW1" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="CX1" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="CX1" s="1" t="s">
+      <c r="CY1" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="CY1" s="1" t="s">
+      <c r="CZ1" s="1" t="s">
         <v>281</v>
-      </c>
-      <c r="CZ1" s="1" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="2" spans="1:104">
@@ -4124,22 +4118,22 @@
         <v>108</v>
       </c>
       <c r="E2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F2" t="s">
         <v>99</v>
       </c>
       <c r="G2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H2" t="s">
         <v>176</v>
       </c>
       <c r="I2" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J2">
-        <v>42.9</v>
+        <v>47.2</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -4169,13 +4163,13 @@
         <v>0</v>
       </c>
       <c r="T2" t="s">
+        <v>336</v>
+      </c>
+      <c r="U2" t="s">
+        <v>337</v>
+      </c>
+      <c r="V2" t="s">
         <v>338</v>
-      </c>
-      <c r="U2" t="s">
-        <v>339</v>
-      </c>
-      <c r="V2" t="s">
-        <v>340</v>
       </c>
       <c r="W2">
         <v>0.5833</v>
@@ -4265,10 +4259,10 @@
         <v>181.2</v>
       </c>
       <c r="AZ2" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA2" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB2">
         <v>96.8</v>
@@ -4355,7 +4349,7 @@
         <v>1.1896</v>
       </c>
       <c r="CD2" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE2">
         <v>858</v>
@@ -4438,25 +4432,25 @@
         <v>108</v>
       </c>
       <c r="E3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G3" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H3" t="s">
         <v>176</v>
       </c>
       <c r="I3" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J3">
-        <v>42.9</v>
+        <v>47.2</v>
       </c>
       <c r="K3">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L3">
         <v>5</v>
@@ -4483,13 +4477,13 @@
         <v>0</v>
       </c>
       <c r="T3" t="s">
+        <v>336</v>
+      </c>
+      <c r="U3" t="s">
         <v>338</v>
       </c>
-      <c r="U3" t="s">
-        <v>340</v>
-      </c>
       <c r="V3" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="W3">
         <v>0.5833</v>
@@ -4579,10 +4573,10 @@
         <v>178.3</v>
       </c>
       <c r="AZ3" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA3" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB3">
         <v>96.2</v>
@@ -4669,7 +4663,7 @@
         <v>1.1896</v>
       </c>
       <c r="CD3" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE3">
         <v>858</v>
@@ -4752,25 +4746,25 @@
         <v>108</v>
       </c>
       <c r="E4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H4" t="s">
         <v>176</v>
       </c>
       <c r="I4" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J4">
-        <v>42.9</v>
+        <v>47.2</v>
       </c>
       <c r="K4">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="L4">
         <v>5</v>
@@ -4797,13 +4791,13 @@
         <v>0</v>
       </c>
       <c r="T4" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U4" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="V4" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="W4">
         <v>0.5833</v>
@@ -4812,7 +4806,7 @@
         <v>6.2</v>
       </c>
       <c r="Y4">
-        <v>93.7</v>
+        <v>93.8</v>
       </c>
       <c r="Z4">
         <v>53.3</v>
@@ -4893,10 +4887,10 @@
         <v>178.2</v>
       </c>
       <c r="AZ4" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA4" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB4">
         <v>96.2</v>
@@ -4983,7 +4977,7 @@
         <v>1.1896</v>
       </c>
       <c r="CD4" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE4">
         <v>858</v>
@@ -5066,25 +5060,25 @@
         <v>108</v>
       </c>
       <c r="E5" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G5" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H5" t="s">
         <v>176</v>
       </c>
       <c r="I5" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J5">
-        <v>42.9</v>
+        <v>47.2</v>
       </c>
       <c r="K5">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="L5">
         <v>5</v>
@@ -5111,13 +5105,13 @@
         <v>0</v>
       </c>
       <c r="T5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U5" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="V5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="W5">
         <v>0.5833</v>
@@ -5207,10 +5201,10 @@
         <v>178</v>
       </c>
       <c r="AZ5" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA5" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB5">
         <v>96.90000000000001</v>
@@ -5297,7 +5291,7 @@
         <v>1.1896</v>
       </c>
       <c r="CD5" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE5">
         <v>858</v>
@@ -5380,25 +5374,25 @@
         <v>109</v>
       </c>
       <c r="E6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F6" t="s">
         <v>100</v>
       </c>
       <c r="G6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H6" t="s">
         <v>177</v>
       </c>
       <c r="I6" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J6">
-        <v>20.7</v>
+        <v>25</v>
       </c>
       <c r="K6">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="L6">
         <v>5</v>
@@ -5425,13 +5419,13 @@
         <v>75</v>
       </c>
       <c r="T6" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U6" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="V6" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="W6">
         <v>0.6667</v>
@@ -5521,10 +5515,10 @@
         <v>232</v>
       </c>
       <c r="AZ6" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BA6" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BB6">
         <v>93.7</v>
@@ -5611,7 +5605,7 @@
         <v>1.1246</v>
       </c>
       <c r="CD6" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE6">
         <v>2633</v>
@@ -5694,25 +5688,25 @@
         <v>109</v>
       </c>
       <c r="E7" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F7" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G7" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H7" t="s">
         <v>177</v>
       </c>
       <c r="I7" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J7">
-        <v>20.7</v>
+        <v>25</v>
       </c>
       <c r="K7">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="L7">
         <v>5</v>
@@ -5739,13 +5733,13 @@
         <v>75</v>
       </c>
       <c r="T7" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U7" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V7" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W7">
         <v>0.6667</v>
@@ -5835,10 +5829,10 @@
         <v>226.9</v>
       </c>
       <c r="AZ7" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BA7" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BB7">
         <v>94.8</v>
@@ -5925,7 +5919,7 @@
         <v>1.1275</v>
       </c>
       <c r="CD7" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE7">
         <v>2530</v>
@@ -6008,25 +6002,25 @@
         <v>109</v>
       </c>
       <c r="E8" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F8" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G8" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H8" t="s">
         <v>177</v>
       </c>
       <c r="I8" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J8">
-        <v>20.7</v>
+        <v>25</v>
       </c>
       <c r="K8">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="L8">
         <v>5</v>
@@ -6053,13 +6047,13 @@
         <v>18.8</v>
       </c>
       <c r="T8" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U8" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V8" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W8">
         <v>0.6667</v>
@@ -6086,7 +6080,7 @@
         <v>-0.2</v>
       </c>
       <c r="AE8" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="AF8">
         <v>78.5</v>
@@ -6149,10 +6143,10 @@
         <v>224.4</v>
       </c>
       <c r="AZ8" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BA8" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BB8">
         <v>78.40000000000001</v>
@@ -6239,7 +6233,7 @@
         <v>1.1338</v>
       </c>
       <c r="CD8" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE8">
         <v>2345</v>
@@ -6322,25 +6316,25 @@
         <v>109</v>
       </c>
       <c r="E9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F9" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="G9" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H9" t="s">
         <v>177</v>
       </c>
       <c r="I9" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J9">
-        <v>20.7</v>
+        <v>25</v>
       </c>
       <c r="K9">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="L9">
         <v>5</v>
@@ -6367,13 +6361,13 @@
         <v>43.8</v>
       </c>
       <c r="T9" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U9" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V9" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W9">
         <v>0.6667</v>
@@ -6400,7 +6394,7 @@
         <v>-0.2</v>
       </c>
       <c r="AE9" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="AF9">
         <v>75.90000000000001</v>
@@ -6463,10 +6457,10 @@
         <v>222.2</v>
       </c>
       <c r="AZ9" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BA9" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BB9">
         <v>96.8</v>
@@ -6553,7 +6547,7 @@
         <v>1.1393</v>
       </c>
       <c r="CD9" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE9">
         <v>2181</v>
@@ -6636,25 +6630,25 @@
         <v>110</v>
       </c>
       <c r="E10" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F10" t="s">
         <v>100</v>
       </c>
       <c r="G10" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H10" t="s">
         <v>178</v>
       </c>
       <c r="I10" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J10">
-        <v>48.3</v>
+        <v>52.6</v>
       </c>
       <c r="K10">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="L10">
         <v>5</v>
@@ -6681,13 +6675,13 @@
         <v>0</v>
       </c>
       <c r="T10" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U10" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="V10" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="W10">
         <v>0.6667</v>
@@ -6777,10 +6771,10 @@
         <v>240.2</v>
       </c>
       <c r="AZ10" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BA10" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BB10">
         <v>79.59999999999999</v>
@@ -6867,7 +6861,7 @@
         <v>1.118</v>
       </c>
       <c r="CD10" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE10">
         <v>2868</v>
@@ -6950,25 +6944,25 @@
         <v>110</v>
       </c>
       <c r="E11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G11" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H11" t="s">
         <v>178</v>
       </c>
       <c r="I11" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J11">
-        <v>48.3</v>
+        <v>52.6</v>
       </c>
       <c r="K11">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="L11">
         <v>5</v>
@@ -6995,13 +6989,13 @@
         <v>0</v>
       </c>
       <c r="T11" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U11" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V11" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W11">
         <v>0.6667</v>
@@ -7028,7 +7022,7 @@
         <v>0.2</v>
       </c>
       <c r="AE11" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="AF11">
         <v>81</v>
@@ -7091,10 +7085,10 @@
         <v>225.2</v>
       </c>
       <c r="AZ11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BA11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BB11">
         <v>72.5</v>
@@ -7181,7 +7175,7 @@
         <v>1.124</v>
       </c>
       <c r="CD11" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE11">
         <v>2674</v>
@@ -7264,25 +7258,25 @@
         <v>110</v>
       </c>
       <c r="E12" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F12" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G12" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H12" t="s">
         <v>178</v>
       </c>
       <c r="I12" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J12">
-        <v>48.3</v>
+        <v>52.6</v>
       </c>
       <c r="K12">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="L12">
         <v>5</v>
@@ -7309,13 +7303,13 @@
         <v>0</v>
       </c>
       <c r="T12" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U12" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V12" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W12">
         <v>0.6667</v>
@@ -7342,7 +7336,7 @@
         <v>0.2</v>
       </c>
       <c r="AE12" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="AF12">
         <v>78.40000000000001</v>
@@ -7405,10 +7399,10 @@
         <v>197.4</v>
       </c>
       <c r="AZ12" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BA12" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BB12">
         <v>90.59999999999999</v>
@@ -7495,7 +7489,7 @@
         <v>1.1285</v>
       </c>
       <c r="CD12" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE12">
         <v>2528</v>
@@ -7578,25 +7572,25 @@
         <v>110</v>
       </c>
       <c r="E13" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F13" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="G13" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H13" t="s">
         <v>178</v>
       </c>
       <c r="I13" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J13">
-        <v>48.3</v>
+        <v>52.6</v>
       </c>
       <c r="K13">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="L13">
         <v>5</v>
@@ -7623,13 +7617,13 @@
         <v>56.2</v>
       </c>
       <c r="T13" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U13" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V13" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W13">
         <v>0.6667</v>
@@ -7656,7 +7650,7 @@
         <v>0.2</v>
       </c>
       <c r="AE13" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="AF13">
         <v>76.5</v>
@@ -7719,10 +7713,10 @@
         <v>177.7</v>
       </c>
       <c r="AZ13" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BA13" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BB13">
         <v>96.3</v>
@@ -7809,7 +7803,7 @@
         <v>1.1318</v>
       </c>
       <c r="CD13" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE13">
         <v>2420</v>
@@ -7892,25 +7886,25 @@
         <v>111</v>
       </c>
       <c r="E14" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F14" t="s">
         <v>100</v>
       </c>
       <c r="G14" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H14" t="s">
         <v>179</v>
       </c>
       <c r="I14" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J14">
-        <v>38.1</v>
+        <v>42.4</v>
       </c>
       <c r="K14">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="L14">
         <v>5</v>
@@ -7937,13 +7931,13 @@
         <v>0</v>
       </c>
       <c r="T14" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U14" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="V14" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="W14">
         <v>0.6667</v>
@@ -8033,10 +8027,10 @@
         <v>240.2</v>
       </c>
       <c r="AZ14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BA14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BB14">
         <v>87</v>
@@ -8123,7 +8117,7 @@
         <v>1.1535</v>
       </c>
       <c r="CD14" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE14">
         <v>1721</v>
@@ -8206,25 +8200,25 @@
         <v>111</v>
       </c>
       <c r="E15" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F15" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G15" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H15" t="s">
         <v>179</v>
       </c>
       <c r="I15" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J15">
-        <v>38.1</v>
+        <v>42.4</v>
       </c>
       <c r="K15">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="L15">
         <v>5</v>
@@ -8251,13 +8245,13 @@
         <v>0</v>
       </c>
       <c r="T15" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U15" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V15" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W15">
         <v>0.6667</v>
@@ -8347,10 +8341,10 @@
         <v>257.9</v>
       </c>
       <c r="AZ15" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BA15" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BB15">
         <v>91.5</v>
@@ -8437,7 +8431,7 @@
         <v>1.1566</v>
       </c>
       <c r="CD15" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE15">
         <v>1640</v>
@@ -8520,25 +8514,25 @@
         <v>111</v>
       </c>
       <c r="E16" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F16" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G16" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H16" t="s">
         <v>179</v>
       </c>
       <c r="I16" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J16">
-        <v>38.1</v>
+        <v>42.4</v>
       </c>
       <c r="K16">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="L16">
         <v>5</v>
@@ -8565,13 +8559,13 @@
         <v>0</v>
       </c>
       <c r="T16" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U16" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V16" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W16">
         <v>0.6667</v>
@@ -8598,7 +8592,7 @@
         <v>-0.2</v>
       </c>
       <c r="AE16" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="AF16">
         <v>81.7</v>
@@ -8661,10 +8655,10 @@
         <v>248.7</v>
       </c>
       <c r="AZ16" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BA16" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BB16">
         <v>92.90000000000001</v>
@@ -8751,7 +8745,7 @@
         <v>1.1591</v>
       </c>
       <c r="CD16" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE16">
         <v>1559</v>
@@ -8834,25 +8828,25 @@
         <v>111</v>
       </c>
       <c r="E17" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="G17" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H17" t="s">
         <v>179</v>
       </c>
       <c r="I17" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J17">
-        <v>38.1</v>
+        <v>42.4</v>
       </c>
       <c r="K17">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="L17">
         <v>5</v>
@@ -8879,13 +8873,13 @@
         <v>0</v>
       </c>
       <c r="T17" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U17" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V17" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W17">
         <v>0.6667</v>
@@ -8912,7 +8906,7 @@
         <v>-0.2</v>
       </c>
       <c r="AE17" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="AF17">
         <v>81.2</v>
@@ -8975,10 +8969,10 @@
         <v>225.4</v>
       </c>
       <c r="AZ17" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BA17" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BB17">
         <v>92.5</v>
@@ -9065,7 +9059,7 @@
         <v>1.1596</v>
       </c>
       <c r="CD17" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE17">
         <v>1526</v>
@@ -9148,25 +9142,25 @@
         <v>112</v>
       </c>
       <c r="E18" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F18" t="s">
         <v>101</v>
       </c>
       <c r="G18" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H18" t="s">
         <v>180</v>
       </c>
       <c r="I18" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J18">
-        <v>46.4</v>
+        <v>50.7</v>
       </c>
       <c r="K18">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="L18">
         <v>5</v>
@@ -9193,13 +9187,13 @@
         <v>0</v>
       </c>
       <c r="T18" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U18" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="V18" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="W18">
         <v>0.75</v>
@@ -9289,10 +9283,10 @@
         <v>152.5</v>
       </c>
       <c r="AZ18" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BA18" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BB18">
         <v>84.7</v>
@@ -9379,7 +9373,7 @@
         <v>1.1494</v>
       </c>
       <c r="CD18" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE18">
         <v>1915</v>
@@ -9462,25 +9456,25 @@
         <v>112</v>
       </c>
       <c r="E19" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F19" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G19" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H19" t="s">
         <v>180</v>
       </c>
       <c r="I19" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J19">
-        <v>46.4</v>
+        <v>50.7</v>
       </c>
       <c r="K19">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="L19">
         <v>5</v>
@@ -9507,13 +9501,13 @@
         <v>0</v>
       </c>
       <c r="T19" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U19" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V19" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W19">
         <v>0.75</v>
@@ -9540,7 +9534,7 @@
         <v>0.5</v>
       </c>
       <c r="AE19" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="AF19">
         <v>80.8</v>
@@ -9603,10 +9597,10 @@
         <v>170.8</v>
       </c>
       <c r="AZ19" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA19" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB19">
         <v>82.90000000000001</v>
@@ -9693,7 +9687,7 @@
         <v>1.1558</v>
       </c>
       <c r="CD19" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE19">
         <v>1712</v>
@@ -9776,25 +9770,25 @@
         <v>112</v>
       </c>
       <c r="E20" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F20" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G20" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H20" t="s">
         <v>180</v>
       </c>
       <c r="I20" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J20">
-        <v>46.4</v>
+        <v>50.7</v>
       </c>
       <c r="K20">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="L20">
         <v>5</v>
@@ -9821,13 +9815,13 @@
         <v>0</v>
       </c>
       <c r="T20" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U20" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V20" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W20">
         <v>0.75</v>
@@ -9854,7 +9848,7 @@
         <v>0.5</v>
       </c>
       <c r="AE20" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="AF20">
         <v>77.59999999999999</v>
@@ -9917,10 +9911,10 @@
         <v>169.7</v>
       </c>
       <c r="AZ20" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA20" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB20">
         <v>82.3</v>
@@ -10007,7 +10001,7 @@
         <v>1.1627</v>
       </c>
       <c r="CD20" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE20">
         <v>1500</v>
@@ -10090,25 +10084,25 @@
         <v>112</v>
       </c>
       <c r="E21" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F21" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G21" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H21" t="s">
         <v>180</v>
       </c>
       <c r="I21" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J21">
-        <v>46.4</v>
+        <v>50.7</v>
       </c>
       <c r="K21">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="L21">
         <v>5</v>
@@ -10135,13 +10129,13 @@
         <v>0</v>
       </c>
       <c r="T21" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U21" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V21" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W21">
         <v>0.75</v>
@@ -10231,10 +10225,10 @@
         <v>169.4</v>
       </c>
       <c r="AZ21" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA21" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB21">
         <v>84.90000000000001</v>
@@ -10321,7 +10315,7 @@
         <v>1.1651</v>
       </c>
       <c r="CD21" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE21">
         <v>1426</v>
@@ -10404,25 +10398,25 @@
         <v>113</v>
       </c>
       <c r="E22" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F22" t="s">
         <v>102</v>
       </c>
       <c r="G22" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="H22" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="I22" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J22">
-        <v>137.2</v>
+        <v>141.4</v>
       </c>
       <c r="K22">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="L22">
         <v>5</v>
@@ -10449,13 +10443,13 @@
         <v>0</v>
       </c>
       <c r="T22" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U22" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V22" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W22">
         <v>0.1667</v>
@@ -10545,10 +10539,10 @@
         <v>227.4</v>
       </c>
       <c r="AZ22" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BA22" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BB22">
         <v>84.8</v>
@@ -10635,7 +10629,7 @@
         <v>1.1156</v>
       </c>
       <c r="CD22" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE22">
         <v>2920</v>
@@ -10718,25 +10712,25 @@
         <v>113</v>
       </c>
       <c r="E23" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F23" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G23" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="H23" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="I23" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J23">
-        <v>137.2</v>
+        <v>141.4</v>
       </c>
       <c r="K23">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="L23">
         <v>5</v>
@@ -10763,13 +10757,13 @@
         <v>0</v>
       </c>
       <c r="T23" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U23" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V23" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W23">
         <v>0.1667</v>
@@ -10859,10 +10853,10 @@
         <v>252</v>
       </c>
       <c r="AZ23" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BA23" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BB23">
         <v>84</v>
@@ -10949,7 +10943,7 @@
         <v>1.1184</v>
       </c>
       <c r="CD23" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE23">
         <v>2826</v>
@@ -11032,25 +11026,25 @@
         <v>113</v>
       </c>
       <c r="E24" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F24" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G24" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="H24" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="I24" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J24">
-        <v>137.2</v>
+        <v>141.4</v>
       </c>
       <c r="K24">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="L24">
         <v>5</v>
@@ -11077,13 +11071,13 @@
         <v>0</v>
       </c>
       <c r="T24" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U24" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V24" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W24">
         <v>0.1667</v>
@@ -11110,7 +11104,7 @@
         <v>2.2</v>
       </c>
       <c r="AE24" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="AF24">
         <v>83.8</v>
@@ -11173,10 +11167,10 @@
         <v>227.8</v>
       </c>
       <c r="AZ24" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BA24" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BB24">
         <v>89.40000000000001</v>
@@ -11263,7 +11257,7 @@
         <v>1.1258</v>
       </c>
       <c r="CD24" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE24">
         <v>2586</v>
@@ -11346,25 +11340,25 @@
         <v>113</v>
       </c>
       <c r="E25" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F25" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G25" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="H25" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="I25" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J25">
-        <v>137.2</v>
+        <v>141.4</v>
       </c>
       <c r="K25">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="L25">
         <v>5</v>
@@ -11391,13 +11385,13 @@
         <v>56.2</v>
       </c>
       <c r="T25" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U25" t="s">
+        <v>345</v>
+      </c>
+      <c r="V25" t="s">
         <v>347</v>
-      </c>
-      <c r="V25" t="s">
-        <v>349</v>
       </c>
       <c r="W25">
         <v>0.1667</v>
@@ -11424,7 +11418,7 @@
         <v>2.2</v>
       </c>
       <c r="AE25" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="AF25">
         <v>78.59999999999999</v>
@@ -11487,10 +11481,10 @@
         <v>182.7</v>
       </c>
       <c r="AZ25" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BA25" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BB25">
         <v>64.90000000000001</v>
@@ -11577,7 +11571,7 @@
         <v>1.1362</v>
       </c>
       <c r="CD25" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE25">
         <v>2248</v>
@@ -11660,25 +11654,25 @@
         <v>114</v>
       </c>
       <c r="E26" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F26" t="s">
         <v>102</v>
       </c>
       <c r="G26" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="H26" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I26" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J26">
-        <v>18.3</v>
+        <v>22.6</v>
       </c>
       <c r="K26">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="L26">
         <v>5</v>
@@ -11705,13 +11699,13 @@
         <v>0</v>
       </c>
       <c r="T26" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U26" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V26" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W26">
         <v>0.1667</v>
@@ -11801,10 +11795,10 @@
         <v>171.2</v>
       </c>
       <c r="AZ26" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA26" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB26">
         <v>84.7</v>
@@ -11891,7 +11885,7 @@
         <v>1.1625</v>
       </c>
       <c r="CD26" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE26">
         <v>1524</v>
@@ -11974,25 +11968,25 @@
         <v>114</v>
       </c>
       <c r="E27" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F27" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G27" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="H27" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I27" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J27">
-        <v>18.3</v>
+        <v>22.6</v>
       </c>
       <c r="K27">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="L27">
         <v>5</v>
@@ -12019,13 +12013,13 @@
         <v>0</v>
       </c>
       <c r="T27" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U27" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V27" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W27">
         <v>0.1667</v>
@@ -12115,10 +12109,10 @@
         <v>175.3</v>
       </c>
       <c r="AZ27" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA27" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB27">
         <v>79.7</v>
@@ -12205,7 +12199,7 @@
         <v>1.1673</v>
       </c>
       <c r="CD27" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE27">
         <v>1375</v>
@@ -12288,25 +12282,25 @@
         <v>114</v>
       </c>
       <c r="E28" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F28" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G28" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="H28" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I28" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J28">
-        <v>18.3</v>
+        <v>22.6</v>
       </c>
       <c r="K28">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="L28">
         <v>5</v>
@@ -12333,13 +12327,13 @@
         <v>0</v>
       </c>
       <c r="T28" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U28" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V28" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W28">
         <v>0.1667</v>
@@ -12429,10 +12423,10 @@
         <v>177.6</v>
       </c>
       <c r="AZ28" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA28" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB28">
         <v>74.59999999999999</v>
@@ -12441,10 +12435,10 @@
         <v>74.59999999999999</v>
       </c>
       <c r="BD28">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="BE28">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="BF28">
         <v>0.1</v>
@@ -12489,7 +12483,7 @@
         <v>3.1</v>
       </c>
       <c r="BT28">
-        <v>-1.6</v>
+        <v>-1.5</v>
       </c>
       <c r="BU28">
         <v>4.5</v>
@@ -12519,7 +12513,7 @@
         <v>1.1706</v>
       </c>
       <c r="CD28" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE28">
         <v>1274</v>
@@ -12602,25 +12596,25 @@
         <v>114</v>
       </c>
       <c r="E29" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F29" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G29" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="H29" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I29" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J29">
-        <v>18.3</v>
+        <v>22.6</v>
       </c>
       <c r="K29">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="L29">
         <v>5</v>
@@ -12647,13 +12641,13 @@
         <v>0</v>
       </c>
       <c r="T29" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U29" t="s">
+        <v>345</v>
+      </c>
+      <c r="V29" t="s">
         <v>347</v>
-      </c>
-      <c r="V29" t="s">
-        <v>349</v>
       </c>
       <c r="W29">
         <v>0.1667</v>
@@ -12680,7 +12674,7 @@
         <v>0.1</v>
       </c>
       <c r="AE29" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="AF29">
         <v>75</v>
@@ -12743,10 +12737,10 @@
         <v>182.7</v>
       </c>
       <c r="AZ29" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BA29" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BB29">
         <v>82.8</v>
@@ -12833,7 +12827,7 @@
         <v>1.1709</v>
       </c>
       <c r="CD29" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE29">
         <v>1266</v>
@@ -12916,25 +12910,25 @@
         <v>115</v>
       </c>
       <c r="E30" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F30" t="s">
         <v>103</v>
       </c>
       <c r="G30" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="H30" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I30" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J30">
-        <v>48.9</v>
+        <v>53.1</v>
       </c>
       <c r="K30">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="L30">
         <v>5</v>
@@ -12961,13 +12955,13 @@
         <v>25</v>
       </c>
       <c r="T30" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U30" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="V30" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="W30">
         <v>0.6667</v>
@@ -13057,10 +13051,10 @@
         <v>231.4</v>
       </c>
       <c r="AZ30" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BA30" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BB30">
         <v>72.40000000000001</v>
@@ -13147,7 +13141,7 @@
         <v>1.1273</v>
       </c>
       <c r="CD30" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE30">
         <v>2475</v>
@@ -13230,25 +13224,25 @@
         <v>115</v>
       </c>
       <c r="E31" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F31" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G31" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="H31" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I31" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J31">
-        <v>48.9</v>
+        <v>53.1</v>
       </c>
       <c r="K31">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="L31">
         <v>5</v>
@@ -13275,13 +13269,13 @@
         <v>25</v>
       </c>
       <c r="T31" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U31" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V31" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W31">
         <v>0.6667</v>
@@ -13308,7 +13302,7 @@
         <v>0.3</v>
       </c>
       <c r="AE31" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="AF31">
         <v>79.8</v>
@@ -13371,10 +13365,10 @@
         <v>252</v>
       </c>
       <c r="AZ31" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BA31" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BB31">
         <v>75.59999999999999</v>
@@ -13461,7 +13455,7 @@
         <v>1.1294</v>
       </c>
       <c r="CD31" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE31">
         <v>2423</v>
@@ -13544,25 +13538,25 @@
         <v>115</v>
       </c>
       <c r="E32" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F32" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="G32" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="H32" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I32" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J32">
-        <v>48.9</v>
+        <v>53.1</v>
       </c>
       <c r="K32">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="L32">
         <v>5</v>
@@ -13589,13 +13583,13 @@
         <v>0</v>
       </c>
       <c r="T32" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U32" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V32" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W32">
         <v>0.6667</v>
@@ -13685,10 +13679,10 @@
         <v>193.5</v>
       </c>
       <c r="AZ32" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BA32" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BB32">
         <v>77.5</v>
@@ -13775,7 +13769,7 @@
         <v>1.1321</v>
       </c>
       <c r="CD32" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE32">
         <v>2350</v>
@@ -13858,25 +13852,25 @@
         <v>115</v>
       </c>
       <c r="E33" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F33" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G33" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="H33" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I33" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J33">
-        <v>48.9</v>
+        <v>53.1</v>
       </c>
       <c r="K33">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="L33">
         <v>5</v>
@@ -13903,13 +13897,13 @@
         <v>0</v>
       </c>
       <c r="T33" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U33" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V33" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W33">
         <v>0.6667</v>
@@ -13999,10 +13993,10 @@
         <v>205</v>
       </c>
       <c r="AZ33" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BA33" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="BB33">
         <v>66</v>
@@ -14089,7 +14083,7 @@
         <v>1.1351</v>
       </c>
       <c r="CD33" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE33">
         <v>2266</v>
@@ -14172,25 +14166,25 @@
         <v>116</v>
       </c>
       <c r="E34" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F34" t="s">
         <v>104</v>
       </c>
       <c r="G34" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="H34" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I34" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J34">
-        <v>18.4</v>
+        <v>22.6</v>
       </c>
       <c r="K34">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="L34">
         <v>5</v>
@@ -14217,13 +14211,13 @@
         <v>0</v>
       </c>
       <c r="T34" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U34" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="V34" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="W34">
         <v>0.75</v>
@@ -14313,10 +14307,10 @@
         <v>257.9</v>
       </c>
       <c r="AZ34" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BA34" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BB34">
         <v>84.90000000000001</v>
@@ -14403,7 +14397,7 @@
         <v>1.1064</v>
       </c>
       <c r="CD34" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE34">
         <v>3245</v>
@@ -14486,25 +14480,25 @@
         <v>116</v>
       </c>
       <c r="E35" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F35" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G35" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="H35" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I35" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J35">
-        <v>18.4</v>
+        <v>22.6</v>
       </c>
       <c r="K35">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="L35">
         <v>5</v>
@@ -14531,13 +14525,13 @@
         <v>0</v>
       </c>
       <c r="T35" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U35" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V35" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W35">
         <v>0.75</v>
@@ -14627,10 +14621,10 @@
         <v>255.7</v>
       </c>
       <c r="AZ35" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BA35" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="BB35">
         <v>86.3</v>
@@ -14717,7 +14711,7 @@
         <v>1.1122</v>
       </c>
       <c r="CD35" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE35">
         <v>3057</v>
@@ -14800,25 +14794,25 @@
         <v>116</v>
       </c>
       <c r="E36" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F36" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G36" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="H36" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I36" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J36">
-        <v>18.4</v>
+        <v>22.6</v>
       </c>
       <c r="K36">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="L36">
         <v>5</v>
@@ -14845,13 +14839,13 @@
         <v>0</v>
       </c>
       <c r="T36" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U36" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V36" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W36">
         <v>0.75</v>
@@ -14941,10 +14935,10 @@
         <v>233.3</v>
       </c>
       <c r="AZ36" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BA36" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BB36">
         <v>88</v>
@@ -15031,7 +15025,7 @@
         <v>1.1174</v>
       </c>
       <c r="CD36" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE36">
         <v>2883</v>
@@ -15114,25 +15108,25 @@
         <v>116</v>
       </c>
       <c r="E37" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F37" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G37" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="H37" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I37" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J37">
-        <v>18.4</v>
+        <v>22.6</v>
       </c>
       <c r="K37">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="L37">
         <v>5</v>
@@ -15159,13 +15153,13 @@
         <v>0</v>
       </c>
       <c r="T37" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U37" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V37" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W37">
         <v>0.75</v>
@@ -15255,10 +15249,10 @@
         <v>233.3</v>
       </c>
       <c r="AZ37" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BA37" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BB37">
         <v>91.8</v>
@@ -15345,7 +15339,7 @@
         <v>1.1217</v>
       </c>
       <c r="CD37" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE37">
         <v>2738</v>
@@ -15428,25 +15422,25 @@
         <v>117</v>
       </c>
       <c r="E38" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F38" t="s">
         <v>105</v>
       </c>
       <c r="G38" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="H38" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I38" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J38">
-        <v>40.4</v>
+        <v>44.6</v>
       </c>
       <c r="K38">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="L38">
         <v>5</v>
@@ -15473,13 +15467,13 @@
         <v>0</v>
       </c>
       <c r="T38" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U38" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="V38" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="W38">
         <v>0.6333</v>
@@ -15569,10 +15563,10 @@
         <v>222.6</v>
       </c>
       <c r="AZ38" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BA38" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BB38">
         <v>93.40000000000001</v>
@@ -15659,7 +15653,7 @@
         <v>1.1604</v>
       </c>
       <c r="CD38" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE38">
         <v>1597</v>
@@ -15742,25 +15736,25 @@
         <v>117</v>
       </c>
       <c r="E39" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F39" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G39" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="H39" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I39" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J39">
-        <v>40.4</v>
+        <v>44.6</v>
       </c>
       <c r="K39">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="L39">
         <v>5</v>
@@ -15787,13 +15781,13 @@
         <v>0</v>
       </c>
       <c r="T39" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U39" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V39" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W39">
         <v>0.6333</v>
@@ -15883,10 +15877,10 @@
         <v>218</v>
       </c>
       <c r="AZ39" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BA39" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BB39">
         <v>93.7</v>
@@ -15973,7 +15967,7 @@
         <v>1.1677</v>
       </c>
       <c r="CD39" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE39">
         <v>1376</v>
@@ -16056,25 +16050,25 @@
         <v>117</v>
       </c>
       <c r="E40" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F40" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G40" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="H40" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I40" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J40">
-        <v>40.4</v>
+        <v>44.6</v>
       </c>
       <c r="K40">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="L40">
         <v>5</v>
@@ -16101,13 +16095,13 @@
         <v>0</v>
       </c>
       <c r="T40" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U40" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V40" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W40">
         <v>0.6333</v>
@@ -16197,10 +16191,10 @@
         <v>195.6</v>
       </c>
       <c r="AZ40" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA40" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB40">
         <v>94.8</v>
@@ -16287,7 +16281,7 @@
         <v>1.1739</v>
       </c>
       <c r="CD40" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE40">
         <v>1190</v>
@@ -16370,25 +16364,25 @@
         <v>117</v>
       </c>
       <c r="E41" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F41" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G41" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="H41" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I41" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J41">
-        <v>40.4</v>
+        <v>44.6</v>
       </c>
       <c r="K41">
-        <v>9.5</v>
+        <v>9.4</v>
       </c>
       <c r="L41">
         <v>5</v>
@@ -16415,13 +16409,13 @@
         <v>0</v>
       </c>
       <c r="T41" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U41" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V41" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W41">
         <v>0.6333</v>
@@ -16511,10 +16505,10 @@
         <v>187.9</v>
       </c>
       <c r="AZ41" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA41" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB41">
         <v>97.5</v>
@@ -16601,7 +16595,7 @@
         <v>1.1784</v>
       </c>
       <c r="CD41" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE41">
         <v>1057</v>
@@ -16684,25 +16678,25 @@
         <v>118</v>
       </c>
       <c r="E42" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F42" t="s">
         <v>106</v>
       </c>
       <c r="G42" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="H42" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I42" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J42">
-        <v>38.9</v>
+        <v>43</v>
       </c>
       <c r="K42">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="L42">
         <v>5</v>
@@ -16729,13 +16723,13 @@
         <v>0</v>
       </c>
       <c r="T42" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U42" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="V42" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="W42">
         <v>0.6667</v>
@@ -16825,10 +16819,10 @@
         <v>211.1</v>
       </c>
       <c r="AZ42" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA42" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB42">
         <v>92.09999999999999</v>
@@ -16915,7 +16909,7 @@
         <v>1.1466</v>
       </c>
       <c r="CD42" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE42">
         <v>2155</v>
@@ -16998,25 +16992,25 @@
         <v>118</v>
       </c>
       <c r="E43" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F43" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G43" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="H43" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I43" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J43">
-        <v>38.9</v>
+        <v>43</v>
       </c>
       <c r="K43">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="L43">
         <v>5</v>
@@ -17043,13 +17037,13 @@
         <v>0</v>
       </c>
       <c r="T43" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U43" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V43" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W43">
         <v>0.6667</v>
@@ -17139,10 +17133,10 @@
         <v>207.2</v>
       </c>
       <c r="AZ43" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA43" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB43">
         <v>92.09999999999999</v>
@@ -17229,7 +17223,7 @@
         <v>1.1572</v>
       </c>
       <c r="CD43" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="CE43">
         <v>1827</v>
@@ -17312,25 +17306,25 @@
         <v>118</v>
       </c>
       <c r="E44" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F44" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G44" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="H44" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I44" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J44">
-        <v>38.9</v>
+        <v>43</v>
       </c>
       <c r="K44">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="L44">
         <v>5</v>
@@ -17357,13 +17351,13 @@
         <v>0</v>
       </c>
       <c r="T44" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U44" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V44" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W44">
         <v>0.6667</v>
@@ -17453,10 +17447,10 @@
         <v>201.8</v>
       </c>
       <c r="AZ44" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA44" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB44">
         <v>94.7</v>
@@ -17543,7 +17537,7 @@
         <v>1.1701</v>
       </c>
       <c r="CD44" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE44">
         <v>1430</v>
@@ -17626,25 +17620,25 @@
         <v>118</v>
       </c>
       <c r="E45" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F45" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G45" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="H45" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I45" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J45">
-        <v>38.9</v>
+        <v>43</v>
       </c>
       <c r="K45">
-        <v>9.5</v>
+        <v>9.4</v>
       </c>
       <c r="L45">
         <v>5</v>
@@ -17671,13 +17665,13 @@
         <v>0</v>
       </c>
       <c r="T45" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U45" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V45" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W45">
         <v>0.6667</v>
@@ -17767,10 +17761,10 @@
         <v>187.4</v>
       </c>
       <c r="AZ45" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BA45" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BB45">
         <v>96.09999999999999</v>
@@ -17857,7 +17851,7 @@
         <v>1.1795</v>
       </c>
       <c r="CD45" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="CE45">
         <v>1148</v>
@@ -17940,25 +17934,25 @@
         <v>119</v>
       </c>
       <c r="E46" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F46" t="s">
         <v>107</v>
       </c>
       <c r="G46" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H46" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I46" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J46">
-        <v>38.4</v>
+        <v>42.5</v>
       </c>
       <c r="K46">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="L46">
         <v>5</v>
@@ -17985,13 +17979,13 @@
         <v>0</v>
       </c>
       <c r="T46" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U46" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="V46" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="W46">
         <v>0.75</v>
@@ -18081,10 +18075,10 @@
         <v>275.4</v>
       </c>
       <c r="AZ46" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BA46" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BB46">
         <v>80.59999999999999</v>
@@ -18171,7 +18165,7 @@
         <v>1.2202</v>
       </c>
       <c r="CD46" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="CE46">
         <v>-42</v>
@@ -18254,25 +18248,25 @@
         <v>119</v>
       </c>
       <c r="E47" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F47" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="G47" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H47" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I47" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J47">
-        <v>38.4</v>
+        <v>42.5</v>
       </c>
       <c r="K47">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="L47">
         <v>5</v>
@@ -18299,13 +18293,13 @@
         <v>0</v>
       </c>
       <c r="T47" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U47" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="V47" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W47">
         <v>0.75</v>
@@ -18395,10 +18389,10 @@
         <v>275.8</v>
       </c>
       <c r="AZ47" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BA47" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="BB47">
         <v>78.8</v>
@@ -18485,7 +18479,7 @@
         <v>1.223</v>
       </c>
       <c r="CD47" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="CE47">
         <v>-118</v>
@@ -18568,25 +18562,25 @@
         <v>119</v>
       </c>
       <c r="E48" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F48" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="G48" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H48" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I48" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J48">
-        <v>38.4</v>
+        <v>42.5</v>
       </c>
       <c r="K48">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="L48">
         <v>5</v>
@@ -18613,13 +18607,13 @@
         <v>0</v>
       </c>
       <c r="T48" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U48" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V48" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="W48">
         <v>0.75</v>
@@ -18709,10 +18703,10 @@
         <v>239.5</v>
       </c>
       <c r="AZ48" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BA48" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="BB48">
         <v>65.8</v>
@@ -18799,7 +18793,7 @@
         <v>1.2246</v>
       </c>
       <c r="CD48" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="CE48">
         <v>-167</v>
@@ -18882,25 +18876,25 @@
         <v>119</v>
       </c>
       <c r="E49" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F49" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G49" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H49" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I49" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J49">
-        <v>38.4</v>
+        <v>42.5</v>
       </c>
       <c r="K49">
-        <v>9.6</v>
+        <v>9.5</v>
       </c>
       <c r="L49">
         <v>5</v>
@@ -18927,13 +18921,13 @@
         <v>56.2</v>
       </c>
       <c r="T49" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="U49" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="V49" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="W49">
         <v>0.75</v>
@@ -19023,10 +19017,10 @@
         <v>211.1</v>
       </c>
       <c r="AZ49" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BA49" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="BB49">
         <v>51.2</v>
@@ -19113,7 +19107,7 @@
         <v>1.2252</v>
       </c>
       <c r="CD49" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="CE49">
         <v>-187</v>
@@ -19870,7 +19864,7 @@
         <v>150</v>
       </c>
       <c r="G13">
-        <v>93</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="H13">
         <v>0</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-27 12:18 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v5_2026_07_27.xlsx
+++ b/mlb_weather_professional_v5_2026_07_27.xlsx
@@ -551,37 +551,37 @@
     <t>HIGH</t>
   </si>
   <si>
-    <t>2026-07-27 12:14:09 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:14:10 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:14:11 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:14:12 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:14:13 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:14:14 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:14:15 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:14:16 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:14:17 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:14:18 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-27 12:14:19 PM PDT</t>
+    <t>2026-07-27 12:17:47 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:17:48 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:17:49 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:17:50 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:17:51 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:17:52 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:17:53 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:17:54 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:17:56 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:17:57 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-27 12:17:58 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -962,37 +962,37 @@
     <t>09:45 PM PDT</t>
   </si>
   <si>
-    <t>2026-07-27 19:14:09 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:14:10 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:14:11 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:14:12 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:14:13 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:14:14 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:14:15 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:14:16 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:14:17 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:14:18 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-27 19:14:19 UTC</t>
+    <t>2026-07-27 19:17:47 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:17:48 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:17:49 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:17:50 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:17:51 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:17:52 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:17:53 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:17:54 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:17:56 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:17:57 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-27 19:17:58 UTC</t>
   </si>
   <si>
     <t>2026-07-27T18:26:57+00:00</t>
@@ -1925,7 +1925,7 @@
         <v>176</v>
       </c>
       <c r="AZ2">
-        <v>47.2</v>
+        <v>50.8</v>
       </c>
       <c r="BA2">
         <v>5</v>
@@ -2014,7 +2014,7 @@
         <v>2.7</v>
       </c>
       <c r="AC3">
-        <v>87.7</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="AD3" t="s">
         <v>164</v>
@@ -2059,7 +2059,7 @@
         <v>167</v>
       </c>
       <c r="AR3">
-        <v>-2.6</v>
+        <v>-2.5</v>
       </c>
       <c r="AS3">
         <v>0</v>
@@ -2083,7 +2083,7 @@
         <v>177</v>
       </c>
       <c r="AZ3">
-        <v>25</v>
+        <v>28.6</v>
       </c>
       <c r="BA3">
         <v>5</v>
@@ -2151,7 +2151,7 @@
         <v>149</v>
       </c>
       <c r="V4">
-        <v>17.7</v>
+        <v>18</v>
       </c>
       <c r="W4">
         <v>60.4</v>
@@ -2229,7 +2229,7 @@
         <v>172</v>
       </c>
       <c r="AV4">
-        <v>22.4</v>
+        <v>22.6</v>
       </c>
       <c r="AW4" t="s">
         <v>173</v>
@@ -2238,10 +2238,10 @@
         <v>5.1</v>
       </c>
       <c r="AY4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AZ4">
-        <v>52.6</v>
+        <v>56.2</v>
       </c>
       <c r="BA4">
         <v>5</v>
@@ -2309,7 +2309,7 @@
         <v>149</v>
       </c>
       <c r="V5">
-        <v>34.7</v>
+        <v>33.1</v>
       </c>
       <c r="W5">
         <v>56.4</v>
@@ -2330,7 +2330,7 @@
         <v>1.9</v>
       </c>
       <c r="AC5">
-        <v>86.2</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="AD5" t="s">
         <v>164</v>
@@ -2387,7 +2387,7 @@
         <v>172</v>
       </c>
       <c r="AV5">
-        <v>33.9</v>
+        <v>33</v>
       </c>
       <c r="AW5" t="s">
         <v>173</v>
@@ -2396,10 +2396,10 @@
         <v>11.1</v>
       </c>
       <c r="AY5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AZ5">
-        <v>42.4</v>
+        <v>46</v>
       </c>
       <c r="BA5">
         <v>5</v>
@@ -2554,10 +2554,10 @@
         <v>11.4</v>
       </c>
       <c r="AY6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AZ6">
-        <v>50.7</v>
+        <v>54.3</v>
       </c>
       <c r="BA6">
         <v>5</v>
@@ -2715,7 +2715,7 @@
         <v>180</v>
       </c>
       <c r="AZ7">
-        <v>141.4</v>
+        <v>145</v>
       </c>
       <c r="BA7">
         <v>5</v>
@@ -2783,7 +2783,7 @@
         <v>149</v>
       </c>
       <c r="V8">
-        <v>27.9</v>
+        <v>28.5</v>
       </c>
       <c r="W8">
         <v>61.5</v>
@@ -2804,7 +2804,7 @@
         <v>3.5</v>
       </c>
       <c r="AC8">
-        <v>89.5</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="AD8" t="s">
         <v>165</v>
@@ -2861,7 +2861,7 @@
         <v>172</v>
       </c>
       <c r="AV8">
-        <v>27.8</v>
+        <v>28.1</v>
       </c>
       <c r="AW8" t="s">
         <v>173</v>
@@ -2873,7 +2873,7 @@
         <v>181</v>
       </c>
       <c r="AZ8">
-        <v>22.6</v>
+        <v>26.2</v>
       </c>
       <c r="BA8">
         <v>5</v>
@@ -2941,7 +2941,7 @@
         <v>149</v>
       </c>
       <c r="V9">
-        <v>32.8</v>
+        <v>31.5</v>
       </c>
       <c r="W9">
         <v>60</v>
@@ -3019,7 +3019,7 @@
         <v>171</v>
       </c>
       <c r="AV9">
-        <v>52.8</v>
+        <v>53.6</v>
       </c>
       <c r="AW9" t="s">
         <v>175</v>
@@ -3031,7 +3031,7 @@
         <v>182</v>
       </c>
       <c r="AZ9">
-        <v>53.1</v>
+        <v>56.7</v>
       </c>
       <c r="BA9">
         <v>5</v>
@@ -3189,7 +3189,7 @@
         <v>183</v>
       </c>
       <c r="AZ10">
-        <v>22.6</v>
+        <v>26.2</v>
       </c>
       <c r="BA10">
         <v>5</v>
@@ -3347,7 +3347,7 @@
         <v>184</v>
       </c>
       <c r="AZ11">
-        <v>44.6</v>
+        <v>48.2</v>
       </c>
       <c r="BA11">
         <v>5</v>
@@ -3505,7 +3505,7 @@
         <v>185</v>
       </c>
       <c r="AZ12">
-        <v>43</v>
+        <v>46.7</v>
       </c>
       <c r="BA12">
         <v>5</v>
@@ -3663,7 +3663,7 @@
         <v>186</v>
       </c>
       <c r="AZ13">
-        <v>42.5</v>
+        <v>46.1</v>
       </c>
       <c r="BA13">
         <v>5</v>
@@ -4133,7 +4133,7 @@
         <v>324</v>
       </c>
       <c r="J2">
-        <v>47.2</v>
+        <v>50.8</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -4447,7 +4447,7 @@
         <v>324</v>
       </c>
       <c r="J3">
-        <v>47.2</v>
+        <v>50.8</v>
       </c>
       <c r="K3">
         <v>0.3</v>
@@ -4761,7 +4761,7 @@
         <v>324</v>
       </c>
       <c r="J4">
-        <v>47.2</v>
+        <v>50.8</v>
       </c>
       <c r="K4">
         <v>1.3</v>
@@ -5075,7 +5075,7 @@
         <v>324</v>
       </c>
       <c r="J5">
-        <v>47.2</v>
+        <v>50.8</v>
       </c>
       <c r="K5">
         <v>2.3</v>
@@ -5389,7 +5389,7 @@
         <v>325</v>
       </c>
       <c r="J6">
-        <v>25</v>
+        <v>28.6</v>
       </c>
       <c r="K6">
         <v>3.4</v>
@@ -5404,7 +5404,7 @@
         <v>2.61</v>
       </c>
       <c r="O6">
-        <v>4.36</v>
+        <v>3.06</v>
       </c>
       <c r="P6">
         <v>4.1</v>
@@ -5431,13 +5431,13 @@
         <v>0.6667</v>
       </c>
       <c r="X6">
-        <v>14.4</v>
+        <v>14</v>
       </c>
       <c r="Y6">
-        <v>87.40000000000001</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="Z6">
-        <v>56.9</v>
+        <v>57</v>
       </c>
       <c r="AA6">
         <v>0.96</v>
@@ -5703,7 +5703,7 @@
         <v>325</v>
       </c>
       <c r="J7">
-        <v>25</v>
+        <v>28.6</v>
       </c>
       <c r="K7">
         <v>4.4</v>
@@ -5718,7 +5718,7 @@
         <v>2.49</v>
       </c>
       <c r="O7">
-        <v>6.18</v>
+        <v>4.69</v>
       </c>
       <c r="P7">
         <v>7.3</v>
@@ -5745,10 +5745,10 @@
         <v>0.6667</v>
       </c>
       <c r="X7">
-        <v>13.2</v>
+        <v>12.7</v>
       </c>
       <c r="Y7">
-        <v>87.90000000000001</v>
+        <v>88.2</v>
       </c>
       <c r="Z7">
         <v>56.4</v>
@@ -5790,7 +5790,7 @@
         <v>77.2</v>
       </c>
       <c r="AM7">
-        <v>33.6</v>
+        <v>34.5</v>
       </c>
       <c r="AN7">
         <v>0.001</v>
@@ -5964,7 +5964,7 @@
         <v>55.2</v>
       </c>
       <c r="CS7">
-        <v>30.9</v>
+        <v>31.4</v>
       </c>
       <c r="CT7" t="s">
         <v>172</v>
@@ -6017,7 +6017,7 @@
         <v>325</v>
       </c>
       <c r="J8">
-        <v>25</v>
+        <v>28.6</v>
       </c>
       <c r="K8">
         <v>5.4</v>
@@ -6032,7 +6032,7 @@
         <v>0.26</v>
       </c>
       <c r="O8">
-        <v>13.29</v>
+        <v>12.63</v>
       </c>
       <c r="P8">
         <v>24.5</v>
@@ -6059,10 +6059,10 @@
         <v>0.6667</v>
       </c>
       <c r="X8">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="Y8">
-        <v>89.3</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="Z8">
         <v>56.1</v>
@@ -6331,7 +6331,7 @@
         <v>325</v>
       </c>
       <c r="J9">
-        <v>25</v>
+        <v>28.6</v>
       </c>
       <c r="K9">
         <v>6.4</v>
@@ -6346,7 +6346,7 @@
         <v>2.36</v>
       </c>
       <c r="O9">
-        <v>21.42</v>
+        <v>21.92</v>
       </c>
       <c r="P9">
         <v>3.6</v>
@@ -6373,10 +6373,10 @@
         <v>0.6667</v>
       </c>
       <c r="X9">
-        <v>15.1</v>
+        <v>15.3</v>
       </c>
       <c r="Y9">
-        <v>85.2</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="Z9">
         <v>55.1</v>
@@ -6636,16 +6636,16 @@
         <v>100</v>
       </c>
       <c r="G10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I10" t="s">
         <v>326</v>
       </c>
       <c r="J10">
-        <v>52.6</v>
+        <v>56.2</v>
       </c>
       <c r="K10">
         <v>3.4</v>
@@ -6660,7 +6660,7 @@
         <v>2.29</v>
       </c>
       <c r="O10">
-        <v>19.25</v>
+        <v>18.96</v>
       </c>
       <c r="P10">
         <v>32</v>
@@ -6687,7 +6687,7 @@
         <v>0.6667</v>
       </c>
       <c r="X10">
-        <v>23.1</v>
+        <v>23</v>
       </c>
       <c r="Y10">
         <v>86.8</v>
@@ -6732,7 +6732,7 @@
         <v>92.2</v>
       </c>
       <c r="AM10">
-        <v>17.7</v>
+        <v>18</v>
       </c>
       <c r="AN10">
         <v>0.005</v>
@@ -6906,7 +6906,7 @@
         <v>58.3</v>
       </c>
       <c r="CS10">
-        <v>22.4</v>
+        <v>22.6</v>
       </c>
       <c r="CT10" t="s">
         <v>172</v>
@@ -6950,16 +6950,16 @@
         <v>289</v>
       </c>
       <c r="G11" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I11" t="s">
         <v>326</v>
       </c>
       <c r="J11">
-        <v>52.6</v>
+        <v>56.2</v>
       </c>
       <c r="K11">
         <v>4.4</v>
@@ -6974,7 +6974,7 @@
         <v>3.63</v>
       </c>
       <c r="O11">
-        <v>21.65</v>
+        <v>20.91</v>
       </c>
       <c r="P11">
         <v>48.9</v>
@@ -7001,10 +7001,10 @@
         <v>0.6667</v>
       </c>
       <c r="X11">
-        <v>28.7</v>
+        <v>28.4</v>
       </c>
       <c r="Y11">
-        <v>85</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="Z11">
         <v>59.2</v>
@@ -7046,7 +7046,7 @@
         <v>84.2</v>
       </c>
       <c r="AM11">
-        <v>17.5</v>
+        <v>18.5</v>
       </c>
       <c r="AN11">
         <v>0.005</v>
@@ -7220,13 +7220,13 @@
         <v>61.5</v>
       </c>
       <c r="CS11">
-        <v>21.1</v>
+        <v>21.6</v>
       </c>
       <c r="CT11" t="s">
         <v>172</v>
       </c>
       <c r="CU11">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="CV11" t="s">
         <v>173</v>
@@ -7264,16 +7264,16 @@
         <v>290</v>
       </c>
       <c r="G12" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H12" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I12" t="s">
         <v>326</v>
       </c>
       <c r="J12">
-        <v>52.6</v>
+        <v>56.2</v>
       </c>
       <c r="K12">
         <v>5.4</v>
@@ -7288,7 +7288,7 @@
         <v>2.84</v>
       </c>
       <c r="O12">
-        <v>18.12</v>
+        <v>17.39</v>
       </c>
       <c r="P12">
         <v>14.4</v>
@@ -7315,10 +7315,10 @@
         <v>0.6667</v>
       </c>
       <c r="X12">
-        <v>22.9</v>
+        <v>22.7</v>
       </c>
       <c r="Y12">
-        <v>88.8</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="Z12">
         <v>57.8</v>
@@ -7360,7 +7360,7 @@
         <v>91.7</v>
       </c>
       <c r="AM12">
-        <v>16.3</v>
+        <v>17.5</v>
       </c>
       <c r="AN12">
         <v>0.002</v>
@@ -7534,7 +7534,7 @@
         <v>64.2</v>
       </c>
       <c r="CS12">
-        <v>18.4</v>
+        <v>19.1</v>
       </c>
       <c r="CT12" t="s">
         <v>173</v>
@@ -7578,16 +7578,16 @@
         <v>291</v>
       </c>
       <c r="G13" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I13" t="s">
         <v>326</v>
       </c>
       <c r="J13">
-        <v>52.6</v>
+        <v>56.2</v>
       </c>
       <c r="K13">
         <v>6.4</v>
@@ -7602,7 +7602,7 @@
         <v>1.4</v>
       </c>
       <c r="O13">
-        <v>10.17</v>
+        <v>10.03</v>
       </c>
       <c r="P13">
         <v>3.9</v>
@@ -7629,7 +7629,7 @@
         <v>0.6667</v>
       </c>
       <c r="X13">
-        <v>13</v>
+        <v>12.9</v>
       </c>
       <c r="Y13">
         <v>91.7</v>
@@ -7674,7 +7674,7 @@
         <v>98.59999999999999</v>
       </c>
       <c r="AM13">
-        <v>14.4</v>
+        <v>15.8</v>
       </c>
       <c r="AN13">
         <v>0</v>
@@ -7848,7 +7848,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="CS13">
-        <v>16.1</v>
+        <v>16.9</v>
       </c>
       <c r="CT13" t="s">
         <v>173</v>
@@ -7892,16 +7892,16 @@
         <v>100</v>
       </c>
       <c r="G14" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H14" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I14" t="s">
         <v>327</v>
       </c>
       <c r="J14">
-        <v>42.4</v>
+        <v>46</v>
       </c>
       <c r="K14">
         <v>3.4</v>
@@ -7916,7 +7916,7 @@
         <v>2.38</v>
       </c>
       <c r="O14">
-        <v>24.39</v>
+        <v>25.48</v>
       </c>
       <c r="P14">
         <v>15.6</v>
@@ -7943,10 +7943,10 @@
         <v>0.6667</v>
       </c>
       <c r="X14">
-        <v>25.3</v>
+        <v>25.7</v>
       </c>
       <c r="Y14">
-        <v>82.5</v>
+        <v>82.3</v>
       </c>
       <c r="Z14">
         <v>56.4</v>
@@ -7988,7 +7988,7 @@
         <v>87.40000000000001</v>
       </c>
       <c r="AM14">
-        <v>34.7</v>
+        <v>33.1</v>
       </c>
       <c r="AN14">
         <v>0.007</v>
@@ -8162,7 +8162,7 @@
         <v>50.6</v>
       </c>
       <c r="CS14">
-        <v>33.9</v>
+        <v>33</v>
       </c>
       <c r="CT14" t="s">
         <v>172</v>
@@ -8206,16 +8206,16 @@
         <v>289</v>
       </c>
       <c r="G15" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I15" t="s">
         <v>327</v>
       </c>
       <c r="J15">
-        <v>42.4</v>
+        <v>46</v>
       </c>
       <c r="K15">
         <v>4.4</v>
@@ -8230,7 +8230,7 @@
         <v>0.91</v>
       </c>
       <c r="O15">
-        <v>23.07</v>
+        <v>24.03</v>
       </c>
       <c r="P15">
         <v>12.1</v>
@@ -8257,10 +8257,10 @@
         <v>0.6667</v>
       </c>
       <c r="X15">
-        <v>18.4</v>
+        <v>18.7</v>
       </c>
       <c r="Y15">
-        <v>87.59999999999999</v>
+        <v>87.5</v>
       </c>
       <c r="Z15">
         <v>58.6</v>
@@ -8302,7 +8302,7 @@
         <v>86</v>
       </c>
       <c r="AM15">
-        <v>18.3</v>
+        <v>16.9</v>
       </c>
       <c r="AN15">
         <v>0.007</v>
@@ -8476,7 +8476,7 @@
         <v>53</v>
       </c>
       <c r="CS15">
-        <v>23.9</v>
+        <v>23.1</v>
       </c>
       <c r="CT15" t="s">
         <v>172</v>
@@ -8520,16 +8520,16 @@
         <v>290</v>
       </c>
       <c r="G16" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H16" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I16" t="s">
         <v>327</v>
       </c>
       <c r="J16">
-        <v>42.4</v>
+        <v>46</v>
       </c>
       <c r="K16">
         <v>5.4</v>
@@ -8544,7 +8544,7 @@
         <v>0.78</v>
       </c>
       <c r="O16">
-        <v>18.76</v>
+        <v>19.51</v>
       </c>
       <c r="P16">
         <v>6.8</v>
@@ -8571,10 +8571,10 @@
         <v>0.6667</v>
       </c>
       <c r="X16">
-        <v>16</v>
+        <v>16.3</v>
       </c>
       <c r="Y16">
-        <v>89.7</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="Z16">
         <v>56.4</v>
@@ -8616,7 +8616,7 @@
         <v>59.8</v>
       </c>
       <c r="AM16">
-        <v>13.4</v>
+        <v>12.3</v>
       </c>
       <c r="AN16">
         <v>0.002</v>
@@ -8790,10 +8790,10 @@
         <v>54.2</v>
       </c>
       <c r="CS16">
-        <v>20.3</v>
+        <v>19.7</v>
       </c>
       <c r="CT16" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="CU16">
         <v>5.6</v>
@@ -8834,16 +8834,16 @@
         <v>291</v>
       </c>
       <c r="G17" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H17" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I17" t="s">
         <v>327</v>
       </c>
       <c r="J17">
-        <v>42.4</v>
+        <v>46</v>
       </c>
       <c r="K17">
         <v>6.4</v>
@@ -8858,7 +8858,7 @@
         <v>0.78</v>
       </c>
       <c r="O17">
-        <v>11.48</v>
+        <v>12.09</v>
       </c>
       <c r="P17">
         <v>13</v>
@@ -8885,10 +8885,10 @@
         <v>0.6667</v>
       </c>
       <c r="X17">
-        <v>13.3</v>
+        <v>13.5</v>
       </c>
       <c r="Y17">
-        <v>90.2</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="Z17">
         <v>55.7</v>
@@ -8930,7 +8930,7 @@
         <v>59</v>
       </c>
       <c r="AM17">
-        <v>9</v>
+        <v>8.1</v>
       </c>
       <c r="AN17">
         <v>0</v>
@@ -9104,7 +9104,7 @@
         <v>53.6</v>
       </c>
       <c r="CS17">
-        <v>17</v>
+        <v>16.5</v>
       </c>
       <c r="CT17" t="s">
         <v>173</v>
@@ -9148,16 +9148,16 @@
         <v>101</v>
       </c>
       <c r="G18" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H18" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I18" t="s">
         <v>328</v>
       </c>
       <c r="J18">
-        <v>50.7</v>
+        <v>54.3</v>
       </c>
       <c r="K18">
         <v>3.5</v>
@@ -9462,16 +9462,16 @@
         <v>292</v>
       </c>
       <c r="G19" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H19" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I19" t="s">
         <v>328</v>
       </c>
       <c r="J19">
-        <v>50.7</v>
+        <v>54.3</v>
       </c>
       <c r="K19">
         <v>4.5</v>
@@ -9776,16 +9776,16 @@
         <v>293</v>
       </c>
       <c r="G20" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H20" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I20" t="s">
         <v>328</v>
       </c>
       <c r="J20">
-        <v>50.7</v>
+        <v>54.3</v>
       </c>
       <c r="K20">
         <v>5.5</v>
@@ -9800,7 +9800,7 @@
         <v>2.11</v>
       </c>
       <c r="O20">
-        <v>20.43</v>
+        <v>20.09</v>
       </c>
       <c r="P20">
         <v>21.8</v>
@@ -9827,10 +9827,10 @@
         <v>0.75</v>
       </c>
       <c r="X20">
-        <v>17.7</v>
+        <v>17.5</v>
       </c>
       <c r="Y20">
-        <v>89.7</v>
+        <v>89.8</v>
       </c>
       <c r="Z20">
         <v>64.59999999999999</v>
@@ -9872,7 +9872,7 @@
         <v>33.2</v>
       </c>
       <c r="AM20">
-        <v>16.6</v>
+        <v>17</v>
       </c>
       <c r="AN20">
         <v>0.001</v>
@@ -10046,7 +10046,7 @@
         <v>63.5</v>
       </c>
       <c r="CS20">
-        <v>18.3</v>
+        <v>18.5</v>
       </c>
       <c r="CT20" t="s">
         <v>173</v>
@@ -10090,16 +10090,16 @@
         <v>294</v>
       </c>
       <c r="G21" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H21" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I21" t="s">
         <v>328</v>
       </c>
       <c r="J21">
-        <v>50.7</v>
+        <v>54.3</v>
       </c>
       <c r="K21">
         <v>6.5</v>
@@ -10114,7 +10114,7 @@
         <v>1.48</v>
       </c>
       <c r="O21">
-        <v>12.3</v>
+        <v>12.21</v>
       </c>
       <c r="P21">
         <v>18.9</v>
@@ -10144,7 +10144,7 @@
         <v>13.4</v>
       </c>
       <c r="Y21">
-        <v>89.59999999999999</v>
+        <v>89.7</v>
       </c>
       <c r="Z21">
         <v>63.2</v>
@@ -10186,7 +10186,7 @@
         <v>65.09999999999999</v>
       </c>
       <c r="AM21">
-        <v>13.5</v>
+        <v>13.7</v>
       </c>
       <c r="AN21">
         <v>0</v>
@@ -10360,7 +10360,7 @@
         <v>64.7</v>
       </c>
       <c r="CS21">
-        <v>15</v>
+        <v>15.1</v>
       </c>
       <c r="CT21" t="s">
         <v>173</v>
@@ -10413,7 +10413,7 @@
         <v>329</v>
       </c>
       <c r="J22">
-        <v>141.4</v>
+        <v>145</v>
       </c>
       <c r="K22">
         <v>3.9</v>
@@ -10428,7 +10428,7 @@
         <v>1.17</v>
       </c>
       <c r="O22">
-        <v>2.47</v>
+        <v>2.41</v>
       </c>
       <c r="P22">
         <v>19.9</v>
@@ -10727,7 +10727,7 @@
         <v>329</v>
       </c>
       <c r="J23">
-        <v>141.4</v>
+        <v>145</v>
       </c>
       <c r="K23">
         <v>4.9</v>
@@ -10742,7 +10742,7 @@
         <v>1.05</v>
       </c>
       <c r="O23">
-        <v>3.9</v>
+        <v>4.15</v>
       </c>
       <c r="P23">
         <v>18.1</v>
@@ -10769,10 +10769,10 @@
         <v>0.1667</v>
       </c>
       <c r="X23">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="Y23">
-        <v>91.3</v>
+        <v>91.2</v>
       </c>
       <c r="Z23">
         <v>67.5</v>
@@ -11041,7 +11041,7 @@
         <v>329</v>
       </c>
       <c r="J24">
-        <v>141.4</v>
+        <v>145</v>
       </c>
       <c r="K24">
         <v>5.9</v>
@@ -11056,7 +11056,7 @@
         <v>0.49</v>
       </c>
       <c r="O24">
-        <v>8.23</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="P24">
         <v>15.9</v>
@@ -11083,10 +11083,10 @@
         <v>0.1667</v>
       </c>
       <c r="X24">
-        <v>5.9</v>
+        <v>6.3</v>
       </c>
       <c r="Y24">
-        <v>90.5</v>
+        <v>90.3</v>
       </c>
       <c r="Z24">
         <v>61.4</v>
@@ -11128,7 +11128,7 @@
         <v>93.5</v>
       </c>
       <c r="AM24">
-        <v>25.6</v>
+        <v>25.8</v>
       </c>
       <c r="AN24">
         <v>0.01</v>
@@ -11302,7 +11302,7 @@
         <v>54.5</v>
       </c>
       <c r="CS24">
-        <v>29.9</v>
+        <v>30</v>
       </c>
       <c r="CT24" t="s">
         <v>172</v>
@@ -11355,7 +11355,7 @@
         <v>329</v>
       </c>
       <c r="J25">
-        <v>141.4</v>
+        <v>145</v>
       </c>
       <c r="K25">
         <v>6.9</v>
@@ -11370,7 +11370,7 @@
         <v>2.47</v>
       </c>
       <c r="O25">
-        <v>6.78</v>
+        <v>5.96</v>
       </c>
       <c r="P25">
         <v>33.5</v>
@@ -11397,10 +11397,10 @@
         <v>0.1667</v>
       </c>
       <c r="X25">
-        <v>26.5</v>
+        <v>26.2</v>
       </c>
       <c r="Y25">
-        <v>77.5</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="Z25">
         <v>53.8</v>
@@ -11669,7 +11669,7 @@
         <v>330</v>
       </c>
       <c r="J26">
-        <v>22.6</v>
+        <v>26.2</v>
       </c>
       <c r="K26">
         <v>3.9</v>
@@ -11684,7 +11684,7 @@
         <v>2.79</v>
       </c>
       <c r="O26">
-        <v>20.53</v>
+        <v>19.68</v>
       </c>
       <c r="P26">
         <v>20</v>
@@ -11711,10 +11711,10 @@
         <v>0.1667</v>
       </c>
       <c r="X26">
-        <v>17.2</v>
+        <v>16.9</v>
       </c>
       <c r="Y26">
-        <v>84.5</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="Z26">
         <v>68.7</v>
@@ -11756,7 +11756,7 @@
         <v>29.4</v>
       </c>
       <c r="AM26">
-        <v>27.9</v>
+        <v>28.5</v>
       </c>
       <c r="AN26">
         <v>0.001</v>
@@ -11930,7 +11930,7 @@
         <v>61.6</v>
       </c>
       <c r="CS26">
-        <v>27.8</v>
+        <v>28.1</v>
       </c>
       <c r="CT26" t="s">
         <v>172</v>
@@ -11983,7 +11983,7 @@
         <v>330</v>
       </c>
       <c r="J27">
-        <v>22.6</v>
+        <v>26.2</v>
       </c>
       <c r="K27">
         <v>4.9</v>
@@ -11998,7 +11998,7 @@
         <v>2.28</v>
       </c>
       <c r="O27">
-        <v>12.47</v>
+        <v>12.07</v>
       </c>
       <c r="P27">
         <v>29.1</v>
@@ -12025,7 +12025,7 @@
         <v>0.1667</v>
       </c>
       <c r="X27">
-        <v>14</v>
+        <v>13.9</v>
       </c>
       <c r="Y27">
         <v>92.09999999999999</v>
@@ -12070,7 +12070,7 @@
         <v>22.4</v>
       </c>
       <c r="AM27">
-        <v>13.4</v>
+        <v>13.8</v>
       </c>
       <c r="AN27">
         <v>0.001</v>
@@ -12244,7 +12244,7 @@
         <v>63.9</v>
       </c>
       <c r="CS27">
-        <v>18.8</v>
+        <v>19</v>
       </c>
       <c r="CT27" t="s">
         <v>173</v>
@@ -12297,7 +12297,7 @@
         <v>330</v>
       </c>
       <c r="J28">
-        <v>22.6</v>
+        <v>26.2</v>
       </c>
       <c r="K28">
         <v>5.9</v>
@@ -12312,7 +12312,7 @@
         <v>2.14</v>
       </c>
       <c r="O28">
-        <v>7.28</v>
+        <v>7.39</v>
       </c>
       <c r="P28">
         <v>34.6</v>
@@ -12384,7 +12384,7 @@
         <v>21.8</v>
       </c>
       <c r="AM28">
-        <v>10.7</v>
+        <v>10.5</v>
       </c>
       <c r="AN28">
         <v>0</v>
@@ -12558,7 +12558,7 @@
         <v>65.40000000000001</v>
       </c>
       <c r="CS28">
-        <v>16.9</v>
+        <v>16.8</v>
       </c>
       <c r="CT28" t="s">
         <v>173</v>
@@ -12611,7 +12611,7 @@
         <v>330</v>
       </c>
       <c r="J29">
-        <v>22.6</v>
+        <v>26.2</v>
       </c>
       <c r="K29">
         <v>6.9</v>
@@ -12626,7 +12626,7 @@
         <v>1.22</v>
       </c>
       <c r="O29">
-        <v>4.11</v>
+        <v>4.22</v>
       </c>
       <c r="P29">
         <v>25.1</v>
@@ -12656,7 +12656,7 @@
         <v>7.9</v>
       </c>
       <c r="Y29">
-        <v>93.7</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="Z29">
         <v>64.5</v>
@@ -12698,7 +12698,7 @@
         <v>59.7</v>
       </c>
       <c r="AM29">
-        <v>7.8</v>
+        <v>8.1</v>
       </c>
       <c r="AN29">
         <v>0</v>
@@ -12872,7 +12872,7 @@
         <v>67.3</v>
       </c>
       <c r="CS29">
-        <v>14.6</v>
+        <v>14.8</v>
       </c>
       <c r="CT29" t="s">
         <v>173</v>
@@ -12925,7 +12925,7 @@
         <v>331</v>
       </c>
       <c r="J30">
-        <v>53.1</v>
+        <v>56.7</v>
       </c>
       <c r="K30">
         <v>4.4</v>
@@ -12940,7 +12940,7 @@
         <v>1.57</v>
       </c>
       <c r="O30">
-        <v>17.58</v>
+        <v>18.34</v>
       </c>
       <c r="P30">
         <v>31.9</v>
@@ -12967,10 +12967,10 @@
         <v>0.6667</v>
       </c>
       <c r="X30">
-        <v>36.2</v>
+        <v>36.5</v>
       </c>
       <c r="Y30">
-        <v>65.90000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="Z30">
         <v>59.1</v>
@@ -13012,7 +13012,7 @@
         <v>77.90000000000001</v>
       </c>
       <c r="AM30">
-        <v>32.8</v>
+        <v>31.5</v>
       </c>
       <c r="AN30">
         <v>0.242</v>
@@ -13186,7 +13186,7 @@
         <v>52.5</v>
       </c>
       <c r="CS30">
-        <v>52</v>
+        <v>51.3</v>
       </c>
       <c r="CT30" t="s">
         <v>171</v>
@@ -13239,7 +13239,7 @@
         <v>331</v>
       </c>
       <c r="J31">
-        <v>53.1</v>
+        <v>56.7</v>
       </c>
       <c r="K31">
         <v>5.4</v>
@@ -13254,7 +13254,7 @@
         <v>0.91</v>
       </c>
       <c r="O31">
-        <v>17.65</v>
+        <v>17.1</v>
       </c>
       <c r="P31">
         <v>24.8</v>
@@ -13281,10 +13281,10 @@
         <v>0.6667</v>
       </c>
       <c r="X31">
-        <v>33.3</v>
+        <v>33.1</v>
       </c>
       <c r="Y31">
-        <v>65.90000000000001</v>
+        <v>66</v>
       </c>
       <c r="Z31">
         <v>64</v>
@@ -13326,7 +13326,7 @@
         <v>73.59999999999999</v>
       </c>
       <c r="AM31">
-        <v>34.2</v>
+        <v>35.6</v>
       </c>
       <c r="AN31">
         <v>0.174</v>
@@ -13500,7 +13500,7 @@
         <v>55.1</v>
       </c>
       <c r="CS31">
-        <v>52.8</v>
+        <v>53.6</v>
       </c>
       <c r="CT31" t="s">
         <v>171</v>
@@ -13553,7 +13553,7 @@
         <v>331</v>
       </c>
       <c r="J32">
-        <v>53.1</v>
+        <v>56.7</v>
       </c>
       <c r="K32">
         <v>6.4</v>
@@ -13568,7 +13568,7 @@
         <v>1.41</v>
       </c>
       <c r="O32">
-        <v>12.8</v>
+        <v>12.73</v>
       </c>
       <c r="P32">
         <v>29.6</v>
@@ -13595,7 +13595,7 @@
         <v>0.6667</v>
       </c>
       <c r="X32">
-        <v>32.9</v>
+        <v>32.8</v>
       </c>
       <c r="Y32">
         <v>65.3</v>
@@ -13640,7 +13640,7 @@
         <v>76.5</v>
       </c>
       <c r="AM32">
-        <v>32</v>
+        <v>32.8</v>
       </c>
       <c r="AN32">
         <v>0.027</v>
@@ -13814,7 +13814,7 @@
         <v>57.6</v>
       </c>
       <c r="CS32">
-        <v>40.3</v>
+        <v>40.7</v>
       </c>
       <c r="CT32" t="s">
         <v>172</v>
@@ -13867,7 +13867,7 @@
         <v>331</v>
       </c>
       <c r="J33">
-        <v>53.1</v>
+        <v>56.7</v>
       </c>
       <c r="K33">
         <v>7.4</v>
@@ -13882,7 +13882,7 @@
         <v>1.97</v>
       </c>
       <c r="O33">
-        <v>7.14</v>
+        <v>6.78</v>
       </c>
       <c r="P33">
         <v>53</v>
@@ -13909,13 +13909,13 @@
         <v>0.6667</v>
       </c>
       <c r="X33">
-        <v>18.4</v>
+        <v>18.3</v>
       </c>
       <c r="Y33">
         <v>82.09999999999999</v>
       </c>
       <c r="Z33">
-        <v>56.1</v>
+        <v>56.2</v>
       </c>
       <c r="AA33">
         <v>1.02</v>
@@ -13954,7 +13954,7 @@
         <v>42.1</v>
       </c>
       <c r="AM33">
-        <v>20.1</v>
+        <v>20.5</v>
       </c>
       <c r="AN33">
         <v>0.008999999999999999</v>
@@ -14128,7 +14128,7 @@
         <v>55.1</v>
       </c>
       <c r="CS33">
-        <v>26.6</v>
+        <v>26.8</v>
       </c>
       <c r="CT33" t="s">
         <v>172</v>
@@ -14181,7 +14181,7 @@
         <v>332</v>
       </c>
       <c r="J34">
-        <v>22.6</v>
+        <v>26.2</v>
       </c>
       <c r="K34">
         <v>4.5</v>
@@ -14196,7 +14196,7 @@
         <v>1.49</v>
       </c>
       <c r="O34">
-        <v>1.69</v>
+        <v>1.32</v>
       </c>
       <c r="P34">
         <v>17.7</v>
@@ -14223,10 +14223,10 @@
         <v>0.75</v>
       </c>
       <c r="X34">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="Y34">
-        <v>89.5</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="Z34">
         <v>74.09999999999999</v>
@@ -14495,7 +14495,7 @@
         <v>332</v>
       </c>
       <c r="J35">
-        <v>22.6</v>
+        <v>26.2</v>
       </c>
       <c r="K35">
         <v>5.5</v>
@@ -14510,7 +14510,7 @@
         <v>1.24</v>
       </c>
       <c r="O35">
-        <v>3.5</v>
+        <v>4.12</v>
       </c>
       <c r="P35">
         <v>17</v>
@@ -14537,13 +14537,13 @@
         <v>0.75</v>
       </c>
       <c r="X35">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="Y35">
-        <v>91</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="Z35">
-        <v>71.59999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="AA35">
         <v>0.96</v>
@@ -14809,7 +14809,7 @@
         <v>332</v>
       </c>
       <c r="J36">
-        <v>22.6</v>
+        <v>26.2</v>
       </c>
       <c r="K36">
         <v>6.5</v>
@@ -14824,7 +14824,7 @@
         <v>0.78</v>
       </c>
       <c r="O36">
-        <v>5</v>
+        <v>4.14</v>
       </c>
       <c r="P36">
         <v>17.5</v>
@@ -14851,10 +14851,10 @@
         <v>0.75</v>
       </c>
       <c r="X36">
-        <v>7.9</v>
+        <v>7.6</v>
       </c>
       <c r="Y36">
-        <v>94.3</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="Z36">
         <v>70.7</v>
@@ -15123,7 +15123,7 @@
         <v>332</v>
       </c>
       <c r="J37">
-        <v>22.6</v>
+        <v>26.2</v>
       </c>
       <c r="K37">
         <v>7.5</v>
@@ -15390,7 +15390,7 @@
         <v>173</v>
       </c>
       <c r="CU37">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="CV37" t="s">
         <v>173</v>
@@ -15437,10 +15437,10 @@
         <v>333</v>
       </c>
       <c r="J38">
-        <v>44.6</v>
+        <v>48.2</v>
       </c>
       <c r="K38">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="L38">
         <v>5</v>
@@ -15751,10 +15751,10 @@
         <v>333</v>
       </c>
       <c r="J39">
-        <v>44.6</v>
+        <v>48.2</v>
       </c>
       <c r="K39">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="L39">
         <v>5</v>
@@ -16065,10 +16065,10 @@
         <v>333</v>
       </c>
       <c r="J40">
-        <v>44.6</v>
+        <v>48.2</v>
       </c>
       <c r="K40">
-        <v>8.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="L40">
         <v>5</v>
@@ -16379,10 +16379,10 @@
         <v>333</v>
       </c>
       <c r="J41">
-        <v>44.6</v>
+        <v>48.2</v>
       </c>
       <c r="K41">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L41">
         <v>5</v>
@@ -16693,7 +16693,7 @@
         <v>334</v>
       </c>
       <c r="J42">
-        <v>43</v>
+        <v>46.7</v>
       </c>
       <c r="K42">
         <v>6.4</v>
@@ -17007,7 +17007,7 @@
         <v>334</v>
       </c>
       <c r="J43">
-        <v>43</v>
+        <v>46.7</v>
       </c>
       <c r="K43">
         <v>7.4</v>
@@ -17321,7 +17321,7 @@
         <v>334</v>
       </c>
       <c r="J44">
-        <v>43</v>
+        <v>46.7</v>
       </c>
       <c r="K44">
         <v>8.4</v>
@@ -17635,7 +17635,7 @@
         <v>334</v>
       </c>
       <c r="J45">
-        <v>43</v>
+        <v>46.7</v>
       </c>
       <c r="K45">
         <v>9.4</v>
@@ -17949,7 +17949,7 @@
         <v>335</v>
       </c>
       <c r="J46">
-        <v>42.5</v>
+        <v>46.1</v>
       </c>
       <c r="K46">
         <v>6.5</v>
@@ -18263,7 +18263,7 @@
         <v>335</v>
       </c>
       <c r="J47">
-        <v>42.5</v>
+        <v>46.1</v>
       </c>
       <c r="K47">
         <v>7.5</v>
@@ -18577,7 +18577,7 @@
         <v>335</v>
       </c>
       <c r="J48">
-        <v>42.5</v>
+        <v>46.1</v>
       </c>
       <c r="K48">
         <v>8.5</v>
@@ -18891,7 +18891,7 @@
         <v>335</v>
       </c>
       <c r="J49">
-        <v>42.5</v>
+        <v>46.1</v>
       </c>
       <c r="K49">
         <v>9.5</v>
@@ -19440,7 +19440,7 @@
         <v>151</v>
       </c>
       <c r="G5">
-        <v>89.5</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="H5">
         <v>7</v>
@@ -19705,7 +19705,7 @@
         <v>150</v>
       </c>
       <c r="G10">
-        <v>87.7</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="H10">
         <v>6</v>
@@ -19758,7 +19758,7 @@
         <v>150</v>
       </c>
       <c r="G11">
-        <v>86.2</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="H11">
         <v>4</v>

</xml_diff>